<commit_message>
Correct scope of the owner cash-to-distribute lines
The quarterly estimate and distribution lines were labelled as covering the
K-1 tax but computed total federal and Arizona income tax on all income,
including the salary and any other household income. Split them: an income
tax line (federal + Arizona), the quarterly estimate off that, and a
distribution line that takes the K-1's pro-rata share — 62,786 rather than
the 100,020 the old label implied.

Also corrected the employee Social Security note, which called the employer
side a matching amount; it additionally carries FUTA and AZ SUTA.

Verified: 1,065 formulas recalculate with zero errors and section 7
reproduces independently.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPxMxc6sHadm8ZMeifvuAx
</commit_message>
<xml_diff>
--- a/Firm_Budget_Forecast_2026.xlsx
+++ b/Firm_Budget_Forecast_2026.xlsx
@@ -458,7 +458,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="492">
   <si>
     <t xml:space="preserve">Onyx Accounting Group, LLC</t>
   </si>
@@ -1730,7 +1730,7 @@
     <t xml:space="preserve">Employee Social Security</t>
   </si>
   <si>
-    <t xml:space="preserve">Withheld from the owner's paycheck. The company pays a matching amount — shown in section 2.</t>
+    <t xml:space="preserve">Withheld from the owner's paycheck. The company separately pays a matching SS and Medicare amount plus FUTA and AZ SUTA — that is the employer tax line in section 2.</t>
   </si>
   <si>
     <t xml:space="preserve">Employee Medicare</t>
@@ -1772,16 +1772,22 @@
     <t xml:space="preserve">NET AFTER-TAX CASH TO OWNER</t>
   </si>
   <si>
+    <t xml:space="preserve">Income tax (federal + Arizona)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total tax less the FICA already withheld from payroll. This is what estimates must cover.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quarterly estimated payment</t>
   </si>
   <si>
-    <t xml:space="preserve">Income tax not covered by payroll withholding, spread over four quarters. Adjust for anything already withheld from salary.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distribution needed to cover the K-1 tax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep at least this much distributable so the owner is not funding firm tax personally.</t>
+    <t xml:space="preserve">Income tax spread over four quarters. Reduce it by any federal or state income tax already withheld from the owner's salary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distribution to cover the tax on K-1 income</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The K-1's pro-rata share of the income tax — the part the salary does not fund. Keep at least this much distributable so the owner is not paying firm tax out of pocket.</t>
   </si>
   <si>
     <t xml:space="preserve">HOW TO READ THIS</t>
@@ -11712,7 +11718,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E81"/>
+  <dimension ref="B1:E82"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -12399,8 +12405,8 @@
         <v>428</v>
       </c>
       <c r="C73" s="57" t="n">
-        <f aca="false">MAX(0,(C64-C60-C61-C62))/4</f>
-        <v>25004.9833258709</v>
+        <f aca="false">C59+C63</f>
+        <v>100019.933303484</v>
       </c>
       <c r="E73" s="19" t="s">
         <v>429</v>
@@ -12411,32 +12417,36 @@
         <v>430</v>
       </c>
       <c r="C74" s="57" t="n">
-        <f aca="false">MAX(0,C64-C60-C61-C62)</f>
-        <v>100019.933303484</v>
+        <f aca="false">C73/4</f>
+        <v>25004.9833258709</v>
       </c>
       <c r="E74" s="19" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B76" s="69" t="s">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B75" s="49" t="s">
         <v>432</v>
       </c>
-      <c r="C76" s="51"/>
-      <c r="D76" s="51"/>
-      <c r="E76" s="51"/>
-    </row>
-    <row r="77" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B77" s="113" t="s">
+      <c r="C75" s="57" t="n">
+        <f aca="false">IF(C51=0,0,C73*C48/C51)</f>
+        <v>62786.1253072978</v>
+      </c>
+      <c r="E75" s="19" t="s">
         <v>433</v>
       </c>
-      <c r="C77" s="113"/>
-      <c r="D77" s="113"/>
-      <c r="E77" s="113"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B77" s="69" t="s">
+        <v>434</v>
+      </c>
+      <c r="C77" s="51"/>
+      <c r="D77" s="51"/>
+      <c r="E77" s="51"/>
     </row>
     <row r="78" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="113" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C78" s="113"/>
       <c r="D78" s="113"/>
@@ -12444,7 +12454,7 @@
     </row>
     <row r="79" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="113" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C79" s="113"/>
       <c r="D79" s="113"/>
@@ -12452,7 +12462,7 @@
     </row>
     <row r="80" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="113" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C80" s="113"/>
       <c r="D80" s="113"/>
@@ -12460,19 +12470,27 @@
     </row>
     <row r="81" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="113" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C81" s="113"/>
       <c r="D81" s="113"/>
       <c r="E81" s="113"/>
     </row>
+    <row r="82" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B82" s="113" t="s">
+        <v>439</v>
+      </c>
+      <c r="C82" s="113"/>
+      <c r="D82" s="113"/>
+      <c r="E82" s="113"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="B77:E77"/>
     <mergeCell ref="B78:E78"/>
     <mergeCell ref="B79:E79"/>
     <mergeCell ref="B80:E80"/>
     <mergeCell ref="B81:E81"/>
+    <mergeCell ref="B82:E82"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12506,45 +12524,45 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="19" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="69" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C6" s="51"/>
       <c r="D6" s="51"/>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="124" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C7" s="125" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D7" s="125"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="52" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="C8" s="125" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D8" s="125"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="52" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C9" s="125" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D9" s="125"/>
     </row>
@@ -12555,62 +12573,62 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="69" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C11" s="51"/>
       <c r="D11" s="51"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="52" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C12" s="125" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="D12" s="125"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="52" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C13" s="125" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D13" s="125"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="52" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C14" s="125" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="D14" s="125"/>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="52" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C15" s="125" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="D15" s="125"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="52" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C16" s="125" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D16" s="125"/>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="52" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C17" s="125" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D17" s="125"/>
     </row>
@@ -12621,35 +12639,35 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="69" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C19" s="51"/>
       <c r="D19" s="127"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="128" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="C20" s="49" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="D20" s="126"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="124" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C21" s="49" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D21" s="129"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="52" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C22" s="49" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="D22" s="126"/>
     </row>
@@ -12658,7 +12676,7 @@
         <v>302</v>
       </c>
       <c r="C23" s="49" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="D23" s="126"/>
     </row>
@@ -12667,7 +12685,7 @@
         <v>303</v>
       </c>
       <c r="C24" s="49" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D24" s="129"/>
     </row>
@@ -12678,14 +12696,14 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="69" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="C26" s="51"/>
       <c r="D26" s="51"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="49" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="132" t="n">
@@ -12695,7 +12713,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="49" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C28" s="49"/>
       <c r="D28" s="132" t="n">
@@ -12705,7 +12723,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="49" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C29" s="49"/>
       <c r="D29" s="132" t="n">
@@ -12715,7 +12733,7 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="49" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C30" s="49"/>
       <c r="D30" s="132" t="n">
@@ -12725,7 +12743,7 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="52" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C31" s="49"/>
       <c r="D31" s="132" t="n">
@@ -12745,7 +12763,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="52" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C33" s="49"/>
       <c r="D33" s="132" t="n">
@@ -12755,7 +12773,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="49" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C34" s="49"/>
       <c r="D34" s="132" t="n">
@@ -12765,7 +12783,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="49" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C35" s="49"/>
       <c r="D35" s="133" t="n">
@@ -12775,7 +12793,7 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="49" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C36" s="49"/>
       <c r="D36" s="133" t="n">
@@ -12785,7 +12803,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="49" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="C37" s="49"/>
       <c r="D37" s="134" t="n">
@@ -12800,80 +12818,80 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="69" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C39" s="51"/>
       <c r="D39" s="51"/>
     </row>
     <row r="40" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C40" s="136" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D40" s="136"/>
     </row>
     <row r="41" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C41" s="136" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="D41" s="136"/>
     </row>
     <row r="42" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C42" s="136" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D42" s="136"/>
     </row>
     <row r="43" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C43" s="136" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D43" s="136"/>
     </row>
     <row r="44" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C44" s="136" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="D44" s="136"/>
     </row>
     <row r="45" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C45" s="136" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D45" s="136"/>
     </row>
     <row r="46" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C46" s="136" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="D46" s="136"/>
     </row>
     <row r="47" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="135" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C47" s="136" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D47" s="136"/>
     </row>

</xml_diff>